<commit_message>
TestPlan Generated and Pushed to Github
</commit_message>
<xml_diff>
--- a/Test_Output/GPIO/TestPlan/GPIO_TestPlan_1.xlsx
+++ b/Test_Output/GPIO/TestPlan/GPIO_TestPlan_1.xlsx
@@ -444,138 +444,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Hidden_Test_Case_Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Hidden_Test_Description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Hidden_Remarks</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Hidden_Test_Steps_Procedure</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Hidden_Impacted_Registers</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Hidden_Validation_Acceptance_Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>gpio_reg_wr_rd_test</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Test performs two phases over CNT=49 registers listed in addr_array[] (MIZAR_GPIO_GP0_GPIO_8..MIZAR_GPIO_GP0_GPIO_39, MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, MIZAR_GPIO_GP0_INTR1_INTR_EN1, MIZAR_GPIO_GP0_INTR1_INTR_STS1, MIZAR_GPIO_GP0_INTR2_INTR_EN1, MIZAR_GPIO_GP0_INTR2_INTR_STS1, MIZAR_GPIO_GPIO_IO_CTRL_GROUP1..4, MIZAR_GPIO_GPIO_DOUT_GROUP1..4, MIZAR_GPIO_GPIO_DIN_GROUP1..4). Phase 1 (chk_rst_val): for i=0..CNT-1, addr=addr_array[i]; if skip_rst_array[i]==1 continue; if read_mask_array[i]==0 continue; data_rd=read_reg(addr); data=(data_rd &amp; 0xfffffffe); if data==default_value_array[i] pass else def_fail_cnt++. Phase 2 (chk_rd_wr): for each j in {0xffffffff,0xaaaaaaaa,0x55555555,0xf5f5f5f5,0xA5A5A5A5,0xffff0000} set data_wr; Write loop: for i=0..CNT-1 if skip_array[i]==1 continue; if write_mask_array[i]==0 continue; write_reg(addr_array[i], (data_wr &amp; write_mask_array[i])); Readback loop: for i=0..CNT-1 if skip_array[i]==1 continue; if write_mask_array[i]==0 continue; if read_mask_array[i]==0 continue; data_rd=(read_reg(addr_array[i]) &amp; read_mask_array[i]); wr_n=(write_mask_array[i] ^ 0xffffffff); exp_val=((data_wr &amp; read_mask_array[i] &amp; write_mask_array[i]) | (wr_n &amp; read_mask_array[i] &amp; default_value_array[i])); if data_rd==exp_val pass else wr_fail_cnt++. test_case() calls chk_rst_val(); chk_rd_wr(); if(def_fail_cnt&gt;0 || wr_fail_cnt&gt;0) finish(1) else finish(0).</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>skip_array[] skips VRRW or otherwise restricted registers for write; skip_rst_array[] skips default-value checks for specific group registers. Note: when reading default values the DIN bit may become 1 if not driven; forcing zero on DIN can drive bit-level selection high, causing read mismatch with expected default.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>["test_case(): call chk_rst_val().","chk_rst_val(): for(i=0;i&lt;CNT;i++){ addr=addr_array[i]; if(skip_rst_array[i]==1) continue; if(read_mask_array[i]==0x00000000) continue; data_rd=read_reg(addr); data=(data_rd &amp; 0xfffffffe); if(data==default_value_array[i]) { } else { def_fail_cnt++; printf failure; } }","Return to test_case(): call chk_rd_wr().","chk_rd_wr(): define chk_val[6]={0xffffffff,0xaaaaaaaa,0x55555555,0xf5f5f5f5,0xA5A5A5A5,0xffff0000}; For each j in 0..5: data_wr=chk_val[j].","Write loop: for(i=0;i&lt;CNT;i++){ addr=addr_array[i]; if(skip_array[i]==1) continue; if(write_mask_array[i]==0x00000000) continue; write_reg(addr,(data_wr &amp; write_mask_array[i])); }","Readback loop: for(i=0;i&lt;CNT;i++){ addr=addr_array[i]; if(skip_array[i]==1) continue; if(write_mask_array[i]==0x00000000) continue; if(read_mask_array[i]==0x00000000) continue; data_rd=(read_reg(addr) &amp; read_mask_array[i]); wr_n=(write_mask_array[i] ^ 0xffffffff); exp_val=((data_wr &amp; read_mask_array[i] &amp; write_mask_array[i]) | (wr_n &amp; read_mask_array[i] &amp; default_value_array[i])); if(data_rd==exp_val){ } else { wr_fail_cnt++; printf failure; } }","Return to test_case(): if(def_fail_cnt&gt;0 || wr_fail_cnt&gt;0) finish(1); else finish(0)."]</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>MIZAR_GPIO_GP0_GPIO_8, MIZAR_GPIO_GP0_GPIO_9, MIZAR_GPIO_GP0_GPIO_10, MIZAR_GPIO_GP0_GPIO_11, MIZAR_GPIO_GP0_GPIO_12, MIZAR_GPIO_GP0_GPIO_13, MIZAR_GPIO_GP0_GPIO_14, MIZAR_GPIO_GP0_GPIO_15, MIZAR_GPIO_GP0_GPIO_16, MIZAR_GPIO_GP0_GPIO_17, MIZAR_GPIO_GP0_GPIO_18, MIZAR_GPIO_GP0_GPIO_19, MIZAR_GPIO_GP0_GPIO_20, MIZAR_GPIO_GP0_GPIO_21, MIZAR_GPIO_GP0_GPIO_22, MIZAR_GPIO_GP0_GPIO_23, MIZAR_GPIO_GP0_GPIO_24, MIZAR_GPIO_GP0_GPIO_25, MIZAR_GPIO_GP0_GPIO_26, MIZAR_GPIO_GP0_GPIO_27, MIZAR_GPIO_GP0_GPIO_28, MIZAR_GPIO_GP0_GPIO_29, MIZAR_GPIO_GP0_GPIO_30, MIZAR_GPIO_GP0_GPIO_31, MIZAR_GPIO_GP0_GPIO_32, MIZAR_GPIO_GP0_GPIO_33, MIZAR_GPIO_GP0_GPIO_34, MIZAR_GPIO_GP0_GPIO_35, MIZAR_GPIO_GP0_GPIO_36, MIZAR_GPIO_GP0_GPIO_37, MIZAR_GPIO_GP0_GPIO_38, MIZAR_GPIO_GP0_GPIO_39, MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, MIZAR_GPIO_GP0_INTR1_INTR_EN1, MIZAR_GPIO_GP0_INTR1_INTR_STS1, MIZAR_GPIO_GP0_INTR2_INTR_EN1, MIZAR_GPIO_GP0_INTR2_INTR_STS1, MIZAR_GPIO_GPIO_IO_CTRL_GROUP1, MIZAR_GPIO_GPIO_IO_CTRL_GROUP2, MIZAR_GPIO_GPIO_IO_CTRL_GROUP3, MIZAR_GPIO_GPIO_IO_CTRL_GROUP4, MIZAR_GPIO_GPIO_DOUT_GROUP1, MIZAR_GPIO_GPIO_DOUT_GROUP2, MIZAR_GPIO_GPIO_DOUT_GROUP3, MIZAR_GPIO_GPIO_DOUT_GROUP4, MIZAR_GPIO_GPIO_DIN_GROUP1, MIZAR_GPIO_GPIO_DIN_GROUP2, MIZAR_GPIO_GPIO_DIN_GROUP3, MIZAR_GPIO_GPIO_DIN_GROUP4</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PASS if def_fail_cnt==0 and wr_fail_cnt==0 at end of test_case(); else FAIL. Default check uses (read_reg(addr) &amp; 0xfffffffe) == default_value_array[i]. Write/read check expects data_rd == ((data_wr &amp; read_mask &amp; write_mask) | ((~write_mask) &amp; read_mask &amp; default_value)).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>test_gpio_negedge_intr_en</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Negative-edge interrupt enable test. test_case(): test_err=0; optionally GIC_EnableIRQ(87) or GIC_EnableIRQ(88) under GPIO0/GPIO1. Enable sysreg interrupt: write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO0_INTR or LSS_SYSREG_INTR_EN1_GPIO1_INTR). Drive all high: write_reg(0xA0243ffc,0xffffffff). Configure pins 8..39: for i=0..31 addr1=MIZAR_GPIO_GP0_GPIO_8+(i4); write_reg(addr1,(1&lt;&lt;20)|(1&lt;&lt;18)|(1&lt;&lt;16)); wait_on(10). For each i=0..31: wr_val=(1&lt;&lt;i); write_reg(MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, wr_val); write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, wr_val); wait_on(10); int_pend=1; write_reg(0xA0243ffc,0xffffffff); wait_on(30); write_reg(0xA0243ffc, ~wr_val); bounded wait: timeout=5000; while(int_pend &amp;&amp; timeout--) wait_on(10); if(timeout==0){ printf timeout; test_err++; }. finish(test_err). Default_IRQHandler(): local_wr=(1&lt;&lt;i); int_pend=0; write_reg(0xA0243ffc,0xffffffff); raddr=MIZAR_GPIO_GP0_GPIO_8+(i4); rdata=read_reg(raddr); if((rdata &amp; 0x1)!=0) test_err++; if((rdata &amp; 0x2)!=0x0){ rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if((rdata_grp &amp; local_wr)==0) test_err++; raddr2=MIZAR_GPIO_GP0_GPIO_8+(i4); write_reg(raddr2,(1&lt;&lt;20)|(1&lt;&lt;16)); write_reg(MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, local_wr); rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if(rdata_grp!=0x0) test_err++; write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO0_INTR or _GPIO1_INTR); GIC_ClearIRQ(87 or 88); } else { test_err++; }</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>The test uses a pad drive at address 0xA0243ffc to synthesize a falling edge per selected bit. A bounded loop with timeout=5000 and wait_on(10) prevents indefinite hang if no interrupt arrives.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>["test_case(): test_err=0.","#ifdef GPIO0: GIC_EnableIRQ(87); #endif; #ifdef GPIO1: GIC_EnableIRQ(88); #endif.","#ifdef GPIO0: write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO0_INTR); #endif.","#ifdef GPIO1: write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO1_INTR); #endif.","write_reg(0xA0243ffc, 0xffffffff);","for(i=0;i&lt;32;i++){ addr1=MIZAR_GPIO_GP0_GPIO_8+(i4); write_reg(addr1, (1u&lt;&lt;20)|(1u&lt;&lt;18)|(1u&lt;&lt;16)); wait_on(10); }","for(i=0;i&lt;32;i++){ wr_val=(1u&lt;&lt;i); write_reg(MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, wr_val); write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, wr_val); wait_on(10); int_pend=1; write_reg(0xA0243ffc, 0xffffffff); wait_on(30); write_reg(0xA0243ffc, ~wr_val); unsigned int timeout=5000; while(int_pend &amp;&amp; timeout--){ wait_on(10);} if(timeout==0){ printf timeout; test_err++; } }","finish(test_err);","Default_IRQHandler(): local_wr=(1u&lt;&lt;i); int_pend=0; write_reg(0xA0243ffc, 0xffffffff); raddr=MIZAR_GPIO_GP0_GPIO_8+(i4); rdata=read_reg(raddr); if((rdata &amp; 0x1)!=0){ test_err++; } if((rdata &amp; 0x2)!=0x0){ rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if((rdata_grp &amp; local_wr)==0){ test_err++; } raddr2=MIZAR_GPIO_GP0_GPIO_8+(i4); write_reg(raddr2, (1u&lt;&lt;20)|(1u&lt;&lt;16)); write_reg(MIZAR_GPIO_GPIO_INTR_RAW_STCLR1, local_wr); rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if(rdata_grp!=0x0){ test_err++; } #ifdef GPIO0: write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO0_INTR); GIC_ClearIRQ(87); #endif; #ifdef GPIO1: write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO1_INTR); GIC_ClearIRQ(88); #endif; } else { test_err++; }"]</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MIZAR_LSS_SYSREG_INTR_EN1, MIZAR_LSS_SYSREG_RAW_STCR1, MIZAR_GPIO_GP0_GPIO_8, MIZAR_GPIO_GP0_INTR1_INTR_EN1, MIZAR_GPIO_GP0_INTR1_INTR_STS1, MIZAR_GPIO_GPIO_INTR_RAW_STCLR1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Per pin: timeout loop must exit by ISR clearing int_pend; in ISR, (rdata &amp; 0x1)==0 (DIN low) and raw bit set ((rdata &amp; 0x2)!=0); group status read MIZAR_GPIO_GP0_INTR1_INTR_STS1 must have the active bit set and become 0 after clearing per-pin and RAW_STCLR1. Sysreg raw clear write is issued; GIC pending IRQ cleared. test_err must remain 0 for PASS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>test_gpio_pedge_all_pads_en</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Positive-edge all‑pads enable test. test_case(): optionally GIC_EnableIRQ(87/88); enable sysreg interrupt via write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO0_INTR or _GPIO1_INTR). For i=0..31: write_reg(MIZAR_GPIO_GP0_GPIO_8+(i4), 0x00020000) to set PEIE (bit17). wait_on(10). Set input mode: write_reg(MIZAR_GPIO_GPIO_IO_CTRL_GROUP1..4, 0x000000FF). wait_on(10). Enable group: write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0xFFFFFFFF). For each i=0..31: write_reg(0xA0243ffc,0x00000000); wait_on(10); int_pend=1; write_reg(0xA0243ffc,0xFFFFFFFF); int timeout=2000; while(int_pend==1 &amp;&amp; --timeout&gt;0){ wait_on(10);} if(timeout==0){ printf timeout; test_err++; break;} write_reg(0xA0243ffc,0x00000000); wait_on(10). finish(test_err). Default_IRQHandler(): wr_val=(1&lt;&lt;i); int_pend=0; rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0x00000000); if((rdata_grp &amp; 0xffffffff)!=0) OK else { printf error; test_err++; }. For j=0..31: write_reg(MIZAR_GPIO_GP0_GPIO_8+(j4),0x00010000) to set ICLR; wait_on(2); rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if(rdata_grp==0x0) OK else { test_err++; }. Clear sysreg raw: write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO0_INTR or _GPIO1_INTR); rdata=read_reg(MIZAR_LSS_SYSREG_RAW_STCR1); if(rdata &amp; bit)!=0 then test_err++; Re‑enable: write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0xFFFFFFFF); GIC_ClearIRQ(87 or 88).</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>External pad drive at 0xA0243ffc is toggled low‑to‑high to generate a rising edge. The wait loop uses timeout=2000 and wait_on(10) per iteration to bound execution time.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>["test_case(): #ifdef GPIO0: GIC_EnableIRQ(87); #endif; #ifdef GPIO1: GIC_EnableIRQ(88); #endif; test_err=0.","#ifdef GPIO0: write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO0_INTR); #endif; #ifdef GPIO1: write_reg(MIZAR_LSS_SYSREG_INTR_EN1, LSS_SYSREG_INTR_EN1_GPIO1_INTR); #endif.","for(i=0;i&lt;32;i++){ write_reg(MIZAR_GPIO_GP0_GPIO_8+(i4), 0x00020000); }","wait_on(10);","write_reg(MIZAR_GPIO_GPIO_IO_CTRL_GROUP1, 0x000000FF); write_reg(MIZAR_GPIO_GPIO_IO_CTRL_GROUP2, 0x000000FF); write_reg(MIZAR_GPIO_GPIO_IO_CTRL_GROUP3, 0x000000FF); write_reg(MIZAR_GPIO_GPIO_IO_CTRL_GROUP4, 0x000000FF);","wait_on(10);","write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0xFFFFFFFF);","for(i=0;i&lt;32;i++){ write_reg(0xA0243ffc, 0x00000000); wait_on(10); int_pend=1; write_reg(0xA0243ffc, 0xFFFFFFFF); int timeout=2000; while((int_pend==1) &amp;&amp; (--timeout&gt;0)){ wait_on(10);} if(timeout==0){ printf timeout; test_err++; break;} write_reg(0xA0243ffc, 0x00000000); wait_on(10); }","finish(test_err);","Default_IRQHandler(): wr_val=(1&lt;&lt;i); int_pend=0; rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0x00000000); if((rdata_grp &amp; 0xffffffff)!=0){ } else { printf error; test_err++; } for(j=0;j&lt;32;j++){ write_reg(MIZAR_GPIO_GP0_GPIO_8+(j4), 0x00010000);} wait_on(2); rdata_grp=read_reg(MIZAR_GPIO_GP0_INTR1_INTR_STS1); if(rdata_grp==0x0){ } else { test_err++; } #ifdef GPIO0: write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO0_INTR); rdata=read_reg(MIZAR_LSS_SYSREG_RAW_STCR1); if((rdata &amp; LSS_SYSREG_RAW_STCR1_GPIO0_INTR)!=0){ test_err++; } #endif; #ifdef GPIO1: write_reg(MIZAR_LSS_SYSREG_RAW_STCR1, LSS_SYSREG_RAW_STCR1_GPIO1_INTR); rdata=read_reg(MIZAR_LSS_SYSREG_RAW_STCR1); if((rdata &amp; LSS_SYSREG_RAW_STCR1_GPIO1_INTR)!=0){ test_err++; } #endif; write_reg(MIZAR_GPIO_GP0_INTR1_INTR_EN1, 0xFFFFFFFF); #ifdef GPIO0: GIC_ClearIRQ(87); #endif; #ifdef GPIO1: GIC_ClearIRQ(88); #endif;"]</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>MIZAR_LSS_SYSREG_INTR_EN1, MIZAR_LSS_SYSREG_RAW_STCR1, MIZAR_GPIO_GP0_GPIO_8, MIZAR_GPIO_GP0_INTR1_INTR_EN1, MIZAR_GPIO_GP0_INTR1_INTR_STS1, MIZAR_GPIO_GPIO_IO_CTRL_GROUP1, MIZAR_GPIO_GPIO_IO_CTRL_GROUP2, MIZAR_GPIO_GPIO_IO_CTRL_GROUP3, MIZAR_GPIO_GPIO_IO_CTRL_GROUP4</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>For each pin: loop must complete without timeout (int_pend cleared in ISR). In ISR: MIZAR_GPIO_GP0_INTR1_INTR_STS1 must be non‑zero on entry; after clearing per‑pin ICLR (write 0x00010000 to each pin reg) the group status must read 0x0. System raw status in MIZAR_LSS_SYSREG_RAW_STCR1 must be cleared (readback with relevant bit 0). test_err must remain 0 to PASS.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>